<commit_message>
add expand & collapse button in viewobjects
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E641F84-C5F1-47CD-B37C-AEABBDA156F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1D06C9-A8CC-46BB-BFAE-B68A2C89BBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8820" yWindow="2030" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3372" uniqueCount="3206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3384" uniqueCount="3218">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24629,6 +24629,49 @@
   </si>
   <si>
     <t>生命值</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ViewObjects.ScrollBottom</t>
+  </si>
+  <si>
+    <t>ViewObjects.CollapseAll</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ViewObjects.ExpandAll</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ViewObjects.ScrollTop</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Expand All</t>
+  </si>
+  <si>
+    <t>Scroll to Top</t>
+  </si>
+  <si>
+    <t>Collapse All</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scroll to Bottom</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>展开全部节点</t>
+  </si>
+  <si>
+    <t>滚动到最上</t>
+  </si>
+  <si>
+    <t>收起全部节点</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>滚动到最下</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -25047,7 +25090,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1126"/>
+  <dimension ref="A1:D1130"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37435,6 +37478,50 @@
         <v>3204</v>
       </c>
     </row>
+    <row r="1127" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1127" s="3" t="s">
+        <v>3207</v>
+      </c>
+      <c r="B1127" s="4" t="s">
+        <v>3216</v>
+      </c>
+      <c r="C1127" s="3" t="s">
+        <v>3212</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1128" s="3" t="s">
+        <v>3208</v>
+      </c>
+      <c r="B1128" s="4" t="s">
+        <v>3214</v>
+      </c>
+      <c r="C1128" s="3" t="s">
+        <v>3210</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1129" s="3" t="s">
+        <v>3209</v>
+      </c>
+      <c r="B1129" s="4" t="s">
+        <v>3215</v>
+      </c>
+      <c r="C1129" s="3" t="s">
+        <v>3211</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1130" s="3" t="s">
+        <v>3206</v>
+      </c>
+      <c r="B1130" s="4" t="s">
+        <v>3217</v>
+      </c>
+      <c r="C1130" s="3" t="s">
+        <v>3213</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add invert selection for multi selection
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1D06C9-A8CC-46BB-BFAE-B68A2C89BBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12B5CED-1A5B-4D26-A569-1E08AB653DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8820" yWindow="2030" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3384" uniqueCount="3218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3387" uniqueCount="3221">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24672,6 +24672,16 @@
   </si>
   <si>
     <t>滚动到最下</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MultiSelectionInvert</t>
+  </si>
+  <si>
+    <t>Invert Selection</t>
+  </si>
+  <si>
+    <t>反向选择</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -25090,7 +25100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1130"/>
+  <dimension ref="A1:D1131"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37522,6 +37532,17 @@
         <v>3213</v>
       </c>
     </row>
+    <row r="1131" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1131" s="3" t="s">
+        <v>3218</v>
+      </c>
+      <c r="B1131" s="4" t="s">
+        <v>3220</v>
+      </c>
+      <c r="C1131" s="3" t="s">
+        <v>3219</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add option to control scroll precision
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12B5CED-1A5B-4D26-A569-1E08AB653DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8519E4D-78E8-4FBC-B2F2-608ABF68CDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8820" yWindow="2030" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3387" uniqueCount="3221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3390" uniqueCount="3224">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24683,6 +24683,16 @@
   <si>
     <t>反向选择</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.ExtFacings.Scroll</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>启用32向的摆放时滚轮调整朝向</t>
+  </si>
+  <si>
+    <t>Allow scroll units into 32 facings when placing</t>
   </si>
 </sst>
 </file>
@@ -25100,7 +25110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1131"/>
+  <dimension ref="A1:D1132"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37543,6 +37553,17 @@
         <v>3219</v>
       </c>
     </row>
+    <row r="1132" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1132" s="3" t="s">
+        <v>3221</v>
+      </c>
+      <c r="B1132" s="4" t="s">
+        <v>3222</v>
+      </c>
+      <c r="C1132" s="3" t="s">
+        <v>3223</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
support 2048 map size
note: sections like waypoints, which are stored as x*1000 + y, remain unchanged yet
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8519E4D-78E8-4FBC-B2F2-608ABF68CDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F2716F1-5AC6-42A0-AED5-14B259AB989F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8820" yWindow="2030" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3390" uniqueCount="3224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3396" uniqueCount="3230">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24693,6 +24693,26 @@
   </si>
   <si>
     <t>Allow scroll units into 32 facings when placing</t>
+  </si>
+  <si>
+    <t>地图宽度和高度必须介于1和2047之间。</t>
+  </si>
+  <si>
+    <t>地图宽度+高度不能超过2048。</t>
+  </si>
+  <si>
+    <t>CreateMap.SizeLimit2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CreateMap.SizeLimit1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The width and height of the map must be between 1 and 2047.</t>
+  </si>
+  <si>
+    <t>Map width plus height cannot exceed 2048.</t>
   </si>
 </sst>
 </file>
@@ -25110,7 +25130,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1132"/>
+  <dimension ref="A1:D1134"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37564,6 +37584,28 @@
         <v>3223</v>
       </c>
     </row>
+    <row r="1133" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1133" s="3" t="s">
+        <v>3227</v>
+      </c>
+      <c r="B1133" s="4" t="s">
+        <v>3224</v>
+      </c>
+      <c r="C1133" s="3" t="s">
+        <v>3228</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1134" s="3" t="s">
+        <v>3226</v>
+      </c>
+      <c r="B1134" s="4" t="s">
+        <v>3225</v>
+      </c>
+      <c r="C1134" s="3" t="s">
+        <v>3229</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>